<commit_message>
chore: update workshop files
</commit_message>
<xml_diff>
--- a/files/dataset-penjualan-finish.xlsx
+++ b/files/dataset-penjualan-finish.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tudemaha/Documents/test-excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89F8BED-75C9-2B4E-A4AF-3F8D184A73EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7575406B-6E77-2743-AA17-C19F3FDA25ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="5" xr2:uid="{6E8E85D2-B145-3848-9EAA-97CE9C9B23EB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{6E8E85D2-B145-3848-9EAA-97CE9C9B23EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Penjualan" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="22" r:id="rId7"/>
+    <pivotCache cacheId="24" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1457" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="538">
   <si>
     <t>ID Pesanan</t>
   </si>
@@ -1667,24 +1667,6 @@
   </si>
   <si>
     <t>Months (Tanggal Pesanan)</t>
-  </si>
-  <si>
-    <t>Jan</t>
-  </si>
-  <si>
-    <t>Feb</t>
-  </si>
-  <si>
-    <t>Mar</t>
-  </si>
-  <si>
-    <t>Apr</t>
-  </si>
-  <si>
-    <t>May</t>
-  </si>
-  <si>
-    <t>Jun</t>
   </si>
   <si>
     <t>Andi Saputra</t>
@@ -1887,9 +1869,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1897,936 +1876,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency [0]" xfId="1" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="196">
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
+  <dxfs count="28">
     <dxf>
       <font>
         <sz val="12"/>
@@ -2994,6 +2052,976 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[dataset-penjualan-finish.xlsx]Pivot3!PivotTable4</c:name>
+    <c:fmtId val="8"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Pivot3!$B$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Pivot3!$A$4:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Andi Saputra</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Budi Santoso</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Citra Dewi</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dewi Lestari</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Eko Prasetyo</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Fitri Handayani</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Gilang Ramadhan</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Hesti Wulandari</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Pivot3!$B$4:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>"Rp"\ #,##0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>134063000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>103587500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>165101000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>138662000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>125618500</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>88647000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>117138000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>142536500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-991F-0F40-ADB7-9A7D7C46744F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="290330768"/>
+        <c:axId val="290332480"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="290330768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="290332480"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="290332480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="&quot;Rp&quot;\ #,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="290330768"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -3071,6 +3099,47 @@
         </xdr:sp>
       </mc:Fallback>
     </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>203200</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>596900</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DC46473A-A22C-2E1A-32EC-CEC9C21A592B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -8133,7 +8202,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8F132739-7F1D-E941-A8B4-F265BA8DE689}" name="PivotTable2" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8F132739-7F1D-E941-A8B4-F265BA8DE689}" name="PivotTable2" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:K26" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="20">
     <pivotField showAll="0"/>
@@ -8846,35 +8915,35 @@
     <dataField name="Sum of Profit" fld="17" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="28">
-    <format dxfId="195">
+    <format dxfId="27">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="194">
+    <format dxfId="26">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="193">
+    <format dxfId="25">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="192">
+    <format dxfId="24">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="191">
+    <format dxfId="23">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="190">
+    <format dxfId="22">
       <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="189">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="188">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="187">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -8890,7 +8959,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="186">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -8906,7 +8975,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="185">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -8921,7 +8990,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="184">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -8935,7 +9004,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="183">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="3">
@@ -8946,38 +9015,38 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="182">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="181">
+    <format dxfId="13">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="180">
+    <format dxfId="12">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="179">
+    <format dxfId="11">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="178">
+    <format dxfId="10">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="177">
+    <format dxfId="9">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="176">
+    <format dxfId="8">
       <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="175">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="174">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="173">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -8993,7 +9062,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="172">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -9009,7 +9078,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="171">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -9024,7 +9093,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="170">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="5" count="1" selected="0">
@@ -9038,7 +9107,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="169">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="3">
@@ -9049,7 +9118,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="168">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -9083,8 +9152,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FADE6E0C-78AE-E44D-B7FC-6E030D9DBE75}" name="PivotTable3" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:D32" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FADE6E0C-78AE-E44D-B7FC-6E030D9DBE75}" name="PivotTable3" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:D17" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="20">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -9223,7 +9292,20 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="10">
+        <item x="0"/>
+        <item x="8"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item x="7"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -9239,7 +9321,7 @@
     <pivotField dataField="1" numFmtId="164" showAll="0"/>
     <pivotField dataField="1" numFmtId="164" showAll="0"/>
     <pivotField showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
+    <pivotField showAll="0" defaultSubtotal="0">
       <items count="14">
         <item x="0"/>
         <item x="1"/>
@@ -9260,9 +9342,9 @@
   </pivotFields>
   <rowFields count="2">
     <field x="2"/>
-    <field x="19"/>
+    <field x="3"/>
   </rowFields>
-  <rowItems count="29">
+  <rowItems count="14">
     <i>
       <x/>
     </i>
@@ -9270,10 +9352,22 @@
       <x v="1"/>
     </i>
     <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
       <x v="2"/>
     </i>
-    <i r="1">
-      <x v="3"/>
+    <i>
+      <x v="2"/>
     </i>
     <i r="1">
       <x v="4"/>
@@ -9281,71 +9375,14 @@
     <i r="1">
       <x v="5"/>
     </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
     <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
       <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
     </i>
     <i r="1">
       <x v="6"/>
     </i>
-    <i>
-      <x v="2"/>
-    </i>
     <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
+      <x v="7"/>
     </i>
     <i t="grand">
       <x/>
@@ -9383,7 +9420,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D9C8D91-3460-8943-B0C3-AAC7598ACB8A}" name="PivotTable4" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D9C8D91-3460-8943-B0C3-AAC7598ACB8A}" name="PivotTable4" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
   <location ref="A3:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="20">
     <pivotField showAll="0"/>
@@ -9615,6 +9652,44 @@
   <dataFields count="1">
     <dataField name="Sum of Profit" fld="17" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -24121,24 +24196,24 @@
       </c>
     </row>
     <row r="222" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A222" s="26" t="s">
+      <c r="A222" s="29" t="s">
         <v>508</v>
       </c>
-      <c r="B222" s="26"/>
-      <c r="C222" s="26"/>
-      <c r="D222" s="26"/>
-      <c r="E222" s="26"/>
-      <c r="F222" s="26"/>
-      <c r="G222" s="26"/>
-      <c r="H222" s="26"/>
-      <c r="I222" s="26"/>
-      <c r="J222" s="26"/>
-      <c r="K222" s="26"/>
-      <c r="L222" s="26"/>
-      <c r="M222" s="26"/>
-      <c r="N222" s="26"/>
-      <c r="O222" s="26"/>
-      <c r="P222" s="26"/>
+      <c r="B222" s="29"/>
+      <c r="C222" s="29"/>
+      <c r="D222" s="29"/>
+      <c r="E222" s="29"/>
+      <c r="F222" s="29"/>
+      <c r="G222" s="29"/>
+      <c r="H222" s="29"/>
+      <c r="I222" s="29"/>
+      <c r="J222" s="29"/>
+      <c r="K222" s="29"/>
+      <c r="L222" s="29"/>
+      <c r="M222" s="29"/>
+      <c r="N222" s="29"/>
+      <c r="O222" s="29"/>
+      <c r="P222" s="29"/>
       <c r="Q222" s="8">
         <f>SUM(Q2:Q221)</f>
         <v>2297485500</v>
@@ -24149,24 +24224,24 @@
       </c>
     </row>
     <row r="223" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A223" s="26" t="s">
+      <c r="A223" s="29" t="s">
         <v>509</v>
       </c>
-      <c r="B223" s="26"/>
-      <c r="C223" s="26"/>
-      <c r="D223" s="26"/>
-      <c r="E223" s="26"/>
-      <c r="F223" s="26"/>
-      <c r="G223" s="26"/>
-      <c r="H223" s="26"/>
-      <c r="I223" s="26"/>
-      <c r="J223" s="26"/>
-      <c r="K223" s="26"/>
-      <c r="L223" s="26"/>
-      <c r="M223" s="26"/>
-      <c r="N223" s="26"/>
-      <c r="O223" s="26"/>
-      <c r="P223" s="26"/>
+      <c r="B223" s="29"/>
+      <c r="C223" s="29"/>
+      <c r="D223" s="29"/>
+      <c r="E223" s="29"/>
+      <c r="F223" s="29"/>
+      <c r="G223" s="29"/>
+      <c r="H223" s="29"/>
+      <c r="I223" s="29"/>
+      <c r="J223" s="29"/>
+      <c r="K223" s="29"/>
+      <c r="L223" s="29"/>
+      <c r="M223" s="29"/>
+      <c r="N223" s="29"/>
+      <c r="O223" s="29"/>
+      <c r="P223" s="29"/>
       <c r="Q223" s="8">
         <f>AVERAGE(Q2:Q222)</f>
         <v>20791723.981900454</v>
@@ -24177,24 +24252,24 @@
       </c>
     </row>
     <row r="224" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A224" s="26" t="s">
+      <c r="A224" s="29" t="s">
         <v>510</v>
       </c>
-      <c r="B224" s="26"/>
-      <c r="C224" s="26"/>
-      <c r="D224" s="26"/>
-      <c r="E224" s="26"/>
-      <c r="F224" s="26"/>
-      <c r="G224" s="26"/>
-      <c r="H224" s="26"/>
-      <c r="I224" s="26"/>
-      <c r="J224" s="26"/>
-      <c r="K224" s="26"/>
-      <c r="L224" s="26"/>
-      <c r="M224" s="26"/>
-      <c r="N224" s="26"/>
-      <c r="O224" s="26"/>
-      <c r="P224" s="26"/>
+      <c r="B224" s="29"/>
+      <c r="C224" s="29"/>
+      <c r="D224" s="29"/>
+      <c r="E224" s="29"/>
+      <c r="F224" s="29"/>
+      <c r="G224" s="29"/>
+      <c r="H224" s="29"/>
+      <c r="I224" s="29"/>
+      <c r="J224" s="29"/>
+      <c r="K224" s="29"/>
+      <c r="L224" s="29"/>
+      <c r="M224" s="29"/>
+      <c r="N224" s="29"/>
+      <c r="O224" s="29"/>
+      <c r="P224" s="29"/>
       <c r="Q224" s="8">
         <f>MAX(Q2:Q221)</f>
         <v>73966000</v>
@@ -24205,24 +24280,24 @@
       </c>
     </row>
     <row r="225" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A225" s="26" t="s">
+      <c r="A225" s="29" t="s">
         <v>511</v>
       </c>
-      <c r="B225" s="26"/>
-      <c r="C225" s="26"/>
-      <c r="D225" s="26"/>
-      <c r="E225" s="26"/>
-      <c r="F225" s="26"/>
-      <c r="G225" s="26"/>
-      <c r="H225" s="26"/>
-      <c r="I225" s="26"/>
-      <c r="J225" s="26"/>
-      <c r="K225" s="26"/>
-      <c r="L225" s="26"/>
-      <c r="M225" s="26"/>
-      <c r="N225" s="26"/>
-      <c r="O225" s="26"/>
-      <c r="P225" s="26"/>
+      <c r="B225" s="29"/>
+      <c r="C225" s="29"/>
+      <c r="D225" s="29"/>
+      <c r="E225" s="29"/>
+      <c r="F225" s="29"/>
+      <c r="G225" s="29"/>
+      <c r="H225" s="29"/>
+      <c r="I225" s="29"/>
+      <c r="J225" s="29"/>
+      <c r="K225" s="29"/>
+      <c r="L225" s="29"/>
+      <c r="M225" s="29"/>
+      <c r="N225" s="29"/>
+      <c r="O225" s="29"/>
+      <c r="P225" s="29"/>
       <c r="Q225" s="8">
         <f>MIN(Q2:Q221)</f>
         <v>62000</v>
@@ -26150,17 +26225,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{322F8BC5-1AC9-9940-A8AB-3CBB68A58EAB}">
-  <dimension ref="A3:D32"/>
+  <dimension ref="A3:D17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>522</v>
       </c>
       <c r="B3" t="s">
@@ -26174,7 +26249,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="27" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="8">
@@ -26188,394 +26263,184 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
-        <v>530</v>
+      <c r="A5" s="28" t="s">
+        <v>40</v>
       </c>
       <c r="B5" s="8">
-        <v>88401000</v>
+        <v>241652000</v>
       </c>
       <c r="C5" s="8">
-        <v>84444500</v>
+        <v>220970500</v>
       </c>
       <c r="D5" s="8">
-        <v>39197500</v>
+        <v>90346500</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="29" t="s">
-        <v>531</v>
+      <c r="A6" s="28" t="s">
+        <v>19</v>
       </c>
       <c r="B6" s="8">
-        <v>58983000</v>
+        <v>187811000</v>
       </c>
       <c r="C6" s="8">
-        <v>58972500</v>
+        <v>178654500</v>
       </c>
       <c r="D6" s="8">
-        <v>29763500</v>
+        <v>83346500</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="29" t="s">
-        <v>532</v>
+      <c r="A7" s="28" t="s">
+        <v>31</v>
       </c>
       <c r="B7" s="8">
-        <v>88573000</v>
+        <v>200229000</v>
       </c>
       <c r="C7" s="8">
-        <v>88515000</v>
+        <v>198161000</v>
       </c>
       <c r="D7" s="8">
-        <v>43248000</v>
+        <v>95063000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
-        <v>533</v>
+      <c r="A8" s="27" t="s">
+        <v>12</v>
       </c>
       <c r="B8" s="8">
-        <v>197900000</v>
+        <v>646419000</v>
       </c>
       <c r="C8" s="8">
-        <v>182206500</v>
+        <v>593624000</v>
       </c>
       <c r="D8" s="8">
-        <v>76654500</v>
+        <v>250236000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="29" t="s">
-        <v>534</v>
+      <c r="A9" s="28" t="s">
+        <v>13</v>
       </c>
       <c r="B9" s="8">
-        <v>164405000</v>
+        <v>280422000</v>
       </c>
       <c r="C9" s="8">
-        <v>154448000</v>
+        <v>265457500</v>
       </c>
       <c r="D9" s="8">
-        <v>66561000</v>
+        <v>116989500</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="29" t="s">
-        <v>535</v>
+      <c r="A10" s="28" t="s">
+        <v>33</v>
       </c>
       <c r="B10" s="8">
-        <v>31430000</v>
+        <v>365997000</v>
       </c>
       <c r="C10" s="8">
-        <v>29199500</v>
+        <v>328166500</v>
       </c>
       <c r="D10" s="8">
-        <v>13331500</v>
+        <v>133246500</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="28" t="s">
-        <v>12</v>
+      <c r="A11" s="27" t="s">
+        <v>25</v>
       </c>
       <c r="B11" s="8">
-        <v>646419000</v>
+        <v>525731000</v>
       </c>
       <c r="C11" s="8">
-        <v>593624000</v>
+        <v>493979000</v>
       </c>
       <c r="D11" s="8">
-        <v>250236000</v>
+        <v>216990000</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="29" t="s">
-        <v>530</v>
+      <c r="A12" s="28" t="s">
+        <v>37</v>
       </c>
       <c r="B12" s="8">
-        <v>166015000</v>
+        <v>250495000</v>
       </c>
       <c r="C12" s="8">
-        <v>151043500</v>
+        <v>222304500</v>
       </c>
       <c r="D12" s="8">
-        <v>63886500</v>
+        <v>88990500</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="29" t="s">
-        <v>531</v>
+      <c r="A13" s="28" t="s">
+        <v>26</v>
       </c>
       <c r="B13" s="8">
-        <v>73025000</v>
+        <v>275236000</v>
       </c>
       <c r="C13" s="8">
-        <v>73022000</v>
+        <v>271674500</v>
       </c>
       <c r="D13" s="8">
-        <v>34028000</v>
+        <v>127999500</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="29" t="s">
-        <v>532</v>
+      <c r="A14" s="27" t="s">
+        <v>22</v>
       </c>
       <c r="B14" s="8">
-        <v>191535000</v>
+        <v>635298000</v>
       </c>
       <c r="C14" s="8">
-        <v>172743500</v>
+        <v>612096500</v>
       </c>
       <c r="D14" s="8">
-        <v>69924500</v>
+        <v>279371500</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="29" t="s">
-        <v>533</v>
+      <c r="A15" s="28" t="s">
+        <v>23</v>
       </c>
       <c r="B15" s="8">
-        <v>86691000</v>
+        <v>263645000</v>
       </c>
       <c r="C15" s="8">
-        <v>71560500</v>
+        <v>250523500</v>
       </c>
       <c r="D15" s="8">
-        <v>23954500</v>
+        <v>110437500</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="29" t="s">
-        <v>534</v>
+      <c r="A16" s="28" t="s">
+        <v>29</v>
       </c>
       <c r="B16" s="8">
-        <v>103858000</v>
+        <v>371653000</v>
       </c>
       <c r="C16" s="8">
-        <v>99994000</v>
+        <v>361573000</v>
       </c>
       <c r="D16" s="8">
-        <v>45316000</v>
+        <v>168934000</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="29" t="s">
-        <v>535</v>
+      <c r="A17" s="27" t="s">
+        <v>523</v>
       </c>
       <c r="B17" s="8">
-        <v>25295000</v>
+        <v>2437140000</v>
       </c>
       <c r="C17" s="8">
-        <v>25260500</v>
+        <v>2297485500</v>
       </c>
       <c r="D17" s="8">
-        <v>13126500</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="8">
-        <v>525731000</v>
-      </c>
-      <c r="C18" s="8">
-        <v>493979000</v>
-      </c>
-      <c r="D18" s="8">
-        <v>216990000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="29" t="s">
-        <v>530</v>
-      </c>
-      <c r="B19" s="8">
-        <v>72234000</v>
-      </c>
-      <c r="C19" s="8">
-        <v>72200500</v>
-      </c>
-      <c r="D19" s="8">
-        <v>34009500</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="29" t="s">
-        <v>531</v>
-      </c>
-      <c r="B20" s="8">
-        <v>48988000</v>
-      </c>
-      <c r="C20" s="8">
-        <v>48973500</v>
-      </c>
-      <c r="D20" s="8">
-        <v>24267500</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="29" t="s">
-        <v>532</v>
-      </c>
-      <c r="B21" s="8">
-        <v>37205000</v>
-      </c>
-      <c r="C21" s="8">
-        <v>37134000</v>
-      </c>
-      <c r="D21" s="8">
-        <v>19466000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="29" t="s">
-        <v>533</v>
-      </c>
-      <c r="B22" s="8">
-        <v>151550000</v>
-      </c>
-      <c r="C22" s="8">
-        <v>137783500</v>
-      </c>
-      <c r="D22" s="8">
-        <v>56926500</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="29" t="s">
-        <v>534</v>
-      </c>
-      <c r="B23" s="8">
-        <v>29968000</v>
-      </c>
-      <c r="C23" s="8">
-        <v>29941500</v>
-      </c>
-      <c r="D23" s="8">
-        <v>14879500</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="29" t="s">
-        <v>535</v>
-      </c>
-      <c r="B24" s="8">
-        <v>185786000</v>
-      </c>
-      <c r="C24" s="8">
-        <v>167946000</v>
-      </c>
-      <c r="D24" s="8">
-        <v>67441000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="8">
-        <v>635298000</v>
-      </c>
-      <c r="C25" s="8">
-        <v>612096500</v>
-      </c>
-      <c r="D25" s="8">
-        <v>279371500</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="29" t="s">
-        <v>530</v>
-      </c>
-      <c r="B26" s="8">
-        <v>139835000</v>
-      </c>
-      <c r="C26" s="8">
-        <v>139785000</v>
-      </c>
-      <c r="D26" s="8">
-        <v>66253000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="29" t="s">
-        <v>531</v>
-      </c>
-      <c r="B27" s="8">
-        <v>42593000</v>
-      </c>
-      <c r="C27" s="8">
-        <v>42582000</v>
-      </c>
-      <c r="D27" s="8">
-        <v>21483000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="29" t="s">
-        <v>532</v>
-      </c>
-      <c r="B28" s="8">
-        <v>174980000</v>
-      </c>
-      <c r="C28" s="8">
-        <v>161909000</v>
-      </c>
-      <c r="D28" s="8">
-        <v>67844000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="29" t="s">
-        <v>533</v>
-      </c>
-      <c r="B29" s="8">
-        <v>91785000</v>
-      </c>
-      <c r="C29" s="8">
-        <v>91736500</v>
-      </c>
-      <c r="D29" s="8">
-        <v>46431500</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="29" t="s">
-        <v>534</v>
-      </c>
-      <c r="B30" s="8">
-        <v>59056000</v>
-      </c>
-      <c r="C30" s="8">
-        <v>59035000</v>
-      </c>
-      <c r="D30" s="8">
-        <v>27969000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="29" t="s">
-        <v>535</v>
-      </c>
-      <c r="B31" s="8">
-        <v>127049000</v>
-      </c>
-      <c r="C31" s="8">
-        <v>117049000</v>
-      </c>
-      <c r="D31" s="8">
-        <v>49391000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="28" t="s">
-        <v>523</v>
-      </c>
-      <c r="B32" s="8">
-        <v>2437140000</v>
-      </c>
-      <c r="C32" s="8">
-        <v>2297485500</v>
-      </c>
-      <c r="D32" s="8">
         <v>1015353500</v>
       </c>
     </row>
@@ -26594,7 +26459,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>529</v>
       </c>
       <c r="B1" t="s">
@@ -26602,7 +26467,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>522</v>
       </c>
       <c r="B3" t="s">
@@ -26610,71 +26475,71 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
-        <v>536</v>
+      <c r="A4" s="27" t="s">
+        <v>530</v>
       </c>
       <c r="B4" s="8">
         <v>134063000</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="28" t="s">
-        <v>537</v>
+      <c r="A5" s="27" t="s">
+        <v>531</v>
       </c>
       <c r="B5" s="8">
         <v>103587500</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
-        <v>538</v>
+      <c r="A6" s="27" t="s">
+        <v>532</v>
       </c>
       <c r="B6" s="8">
         <v>165101000</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="28" t="s">
-        <v>539</v>
+      <c r="A7" s="27" t="s">
+        <v>533</v>
       </c>
       <c r="B7" s="8">
         <v>138662000</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
-        <v>540</v>
+      <c r="A8" s="27" t="s">
+        <v>534</v>
       </c>
       <c r="B8" s="8">
         <v>125618500</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="28" t="s">
-        <v>541</v>
+      <c r="A9" s="27" t="s">
+        <v>535</v>
       </c>
       <c r="B9" s="8">
         <v>88647000</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="28" t="s">
-        <v>542</v>
+      <c r="A10" s="27" t="s">
+        <v>536</v>
       </c>
       <c r="B10" s="8">
         <v>117138000</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="28" t="s">
-        <v>543</v>
+      <c r="A11" s="27" t="s">
+        <v>537</v>
       </c>
       <c r="B11" s="8">
         <v>142536500</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="27" t="s">
         <v>523</v>
       </c>
       <c r="B12" s="8">
@@ -26683,5 +26548,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>